<commit_message>
Cronograma INS+EL Rev.1: entrega progresiva de instrumentos + contexto 3D
- Entrega progresiva: Fase 1 (valvulas + instrumentos en linea, 920) primero;
  Fase 2 (resto montaje especifico, 1.878) progresiva desde FEB-2027
- Desdobla recepcion/banco y montaje en Fase 1 (con caneria) y Fase 2
- Agrega pagina de contexto de planta (vista 3D) renderizada desde el PDF original
- RFSU 20-DIC-2027 confirmado como hito gobernante
</commit_message>
<xml_diff>
--- a/Constructibilidad/Análisis generados/Cronograma_INS_EL_CPF2.xlsx
+++ b/Constructibilidad/Análisis generados/Cronograma_INS_EL_CPF2.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -591,23 +591,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M4a</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>▼ Entrega instrumentos AESA (a banco)</t>
+          <t>▼ Entrega instrum. Fase 1 (válvulas + en línea)</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46402</v>
+        <v>46371</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>~1.163 instr AESA</t>
+          <t>920 en línea (válv 485+elem 435)</t>
         </is>
       </c>
     </row>
@@ -619,23 +619,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4b</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>▼ Llegada Cables EL a sitio</t>
+          <t>▼ Entrega instrum. Fase 2 (resto, progresiva)</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46446</v>
+        <v>46433</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>513 c / 81.231 m</t>
+          <t>1.878 montaje específico</t>
         </is>
       </c>
     </row>
@@ -647,27 +647,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>★ Inicio campo PCS — Sala INS (Sala 7)</t>
+          <t>▼ Llegada Cables EL a sitio</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46463</v>
+        <v>46446</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>ancla IN</t>
+          <t>513 c / 81.231 m</t>
         </is>
       </c>
     </row>
@@ -679,23 +675,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>M6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>★ Llegada SE#4 (con PMS-101)</t>
+          <t>★ Inicio campo PCS — Sala INS (Sala 7)</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46485</v>
+        <v>46463</v>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ancla EL</t>
+          <t>ancla IN</t>
         </is>
       </c>
     </row>
@@ -707,75 +707,71 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>M7</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>★ Llegada SE#3 (con PMS-001)</t>
+          <t>★ Llegada SE#4 (con PMS-101)</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46521</v>
+        <v>46485</v>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ancla EL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Provisión</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>★ Llegada SE#3 (con PMS-001)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>46521</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
         <is>
           <t>SÍ</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>ancla EL · ruta crítica</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>INSTRUMENTACIÓN (IN) — PCS / SIS / F&amp;G</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Instrumentación</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>I1</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Canalizaciones / conduit instrumentación</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>46354</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>46418</v>
-      </c>
-      <c r="F12" t="n">
-        <v>65</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>bandeja+conduit IN</t>
-        </is>
-      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -785,31 +781,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>I2</t>
+          <t>I1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tendido cables IN — señal 1P/1T (≈609 c)</t>
+          <t>Canalizaciones / conduit instrumentación</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46419</v>
+        <v>46354</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>46446</v>
+        <v>46418</v>
       </c>
       <c r="F13" t="n">
-        <v>28</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>~31.600 m</t>
+          <t>bandeja+conduit IN</t>
         </is>
       </c>
     </row>
@@ -821,22 +813,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>I3</t>
+          <t>I2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tendido cables IN — multipar/terna (≈260 c)</t>
+          <t>Tendido cables IN — señal 1P/1T (≈609 c)</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46428</v>
+        <v>46419</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>46460</v>
+        <v>46446</v>
       </c>
       <c r="F14" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -845,7 +837,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>~30.000 m · 5-6 cuad.</t>
+          <t>~31.600 m</t>
         </is>
       </c>
     </row>
@@ -857,27 +849,31 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>I3</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tendido cables IN — FO / FTP (16 c)</t>
+          <t>Tendido cables IN — multipar/terna (≈260 c)</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46447</v>
+        <v>46428</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>46460</v>
       </c>
       <c r="F15" t="n">
-        <v>14</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
+        <v>33</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>~3.300 m</t>
+          <t>~30.000 m · 5-6 cuad.</t>
         </is>
       </c>
     </row>
@@ -889,27 +885,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>I5</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Recepción + prueba en banco instrumentos (calib.)</t>
+          <t>Tendido cables IN — FO / FTP (16 c)</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46402</v>
+        <v>46447</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>46477</v>
+        <v>46460</v>
       </c>
       <c r="F16" t="n">
-        <v>76</v>
+        <v>14</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>~1.163 instr · pre-montaje</t>
+          <t>~3.300 m</t>
         </is>
       </c>
     </row>
@@ -921,27 +917,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>I6</t>
+          <t>I5a</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Montaje instrumentos en campo — AESA</t>
+          <t>Recepción + banco Fase 1 (válvulas/PSV + en línea)</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46447</v>
+        <v>46371</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>46568</v>
+        <v>46446</v>
       </c>
       <c r="F17" t="n">
-        <v>122</v>
+        <v>76</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1.163 instr (7 típicos)</t>
+          <t>en línea · pre-montaje</t>
         </is>
       </c>
     </row>
@@ -953,31 +949,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>I7</t>
+          <t>I6a</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Conexionado IN — campo→JB→Sala INS</t>
+          <t>Montaje instrum. en línea — AESA (con cañería)</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46463</v>
+        <v>46402</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>46599</v>
+        <v>46507</v>
       </c>
       <c r="F18" t="n">
-        <v>137</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>15.752 puntas</t>
+          <t>válvulas + elementos</t>
         </is>
       </c>
     </row>
@@ -989,143 +981,143 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>I8</t>
+          <t>I5b</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Loop check IN (sensor→JB→PCS/SIS)</t>
+          <t>Recepción + banco Fase 2 (resto instrumentos)</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46539</v>
+        <v>46433</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>46619</v>
+        <v>46522</v>
       </c>
       <c r="F19" t="n">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>~885 lazos</t>
+          <t>montaje específico</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>ELECTRICIDAD (EL) — Potencia / Control</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr"/>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Instrumentación</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>I6b</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Montaje instrum. montaje específico — AESA</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>46461</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>46568</v>
+      </c>
+      <c r="F20" t="n">
+        <v>108</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>transmisores/sw/F&amp;G</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Electricidad</t>
+          <t>Instrumentación</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>I7</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Bandejas portacables principales</t>
+          <t>Conexionado IN — campo→JB→Sala INS</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46447</v>
+        <v>46463</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>46482</v>
+        <v>46599</v>
       </c>
       <c r="F21" t="n">
-        <v>36</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
+        <v>137</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>MC1/MC2/MC3</t>
+          <t>15.752 puntas</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Electricidad</t>
+          <t>Instrumentación</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>I8</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Tendido EL — Potencia BT Grande ≥35mm²</t>
+          <t>Loop check IN (sensor→JB→PCS/SIS)</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46447</v>
+        <v>46539</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>46495</v>
+        <v>46619</v>
       </c>
       <c r="F22" t="n">
-        <v>49</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>104 c / 17.470 m ★</t>
+          <t>~885 lazos</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Electricidad</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>E3</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Tendido EL — Potencia BT Med/Peq</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>46461</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>46503</v>
-      </c>
-      <c r="F23" t="n">
-        <v>43</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>198 c / 33.125 m</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>ELECTRICIDAD (EL) — Potencia / Control</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1135,27 +1127,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tendido EL — Control y Señales</t>
+          <t>Bandejas portacables principales</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46461</v>
+        <v>46447</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>46520</v>
+        <v>46482</v>
       </c>
       <c r="F24" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>192 c / 28.126 m</t>
+          <t>MC1/MC2/MC3</t>
         </is>
       </c>
     </row>
@@ -1167,27 +1159,31 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tendido EL — Potencia MT 6,6/13,2kV</t>
+          <t>Tendido EL — Potencia BT Grande ≥35mm²</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46517</v>
+        <v>46447</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>46545</v>
+        <v>46495</v>
       </c>
       <c r="F25" t="n">
-        <v>29</v>
-      </c>
-      <c r="G25" t="inlineStr"/>
+        <v>49</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>18 c / 2.110 m · cert. ABB</t>
+          <t>104 c / 17.470 m ★</t>
         </is>
       </c>
     </row>
@@ -1199,27 +1195,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Armado shelter SE#4 (módulos en campo)</t>
+          <t>Tendido EL — Potencia BT Med/Peq</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46485</v>
+        <v>46461</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>46499</v>
+        <v>46503</v>
       </c>
       <c r="F26" t="n">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>14 d</t>
+          <t>198 c / 33.125 m</t>
         </is>
       </c>
     </row>
@@ -1231,27 +1227,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Montaje CCMs / celdas MT / motores</t>
+          <t>Tendido EL — Control y Señales</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46491</v>
+        <v>46461</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>46531</v>
+        <v>46520</v>
       </c>
       <c r="F27" t="n">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>37 tabl · 79 motores</t>
+          <t>192 c / 28.126 m</t>
         </is>
       </c>
     </row>
@@ -1263,31 +1259,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>E8</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Armado shelter SE#3 (módulos en campo)</t>
+          <t>Tendido EL — Potencia MT 6,6/13,2kV</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46521</v>
+        <v>46517</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>46541</v>
+        <v>46545</v>
       </c>
       <c r="F28" t="n">
-        <v>21</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>21 d · ruta crítica</t>
+          <t>18 c / 2.110 m · cert. ABB</t>
         </is>
       </c>
     </row>
@@ -1299,27 +1291,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>E9</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Conexionado EL — Sector SE#4</t>
+          <t>Armado shelter SE#4 (módulos en campo)</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46500</v>
+        <v>46485</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>46550</v>
+        <v>46499</v>
       </c>
       <c r="F29" t="n">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>puntas BT+control S4</t>
+          <t>14 d</t>
         </is>
       </c>
     </row>
@@ -1331,27 +1323,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Conexionado EL — Terminaciones MT (36 ext.)</t>
+          <t>Montaje CCMs / celdas MT / motores</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46545</v>
+        <v>46491</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>46573</v>
+        <v>46531</v>
       </c>
       <c r="F30" t="n">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
-          <t>técnicos cert. ABB</t>
+          <t>37 tabl · 79 motores</t>
         </is>
       </c>
     </row>
@@ -1363,108 +1355,122 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Conexionado EL — Sector SE#3</t>
+          <t>Armado shelter SE#3 (módulos en campo)</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46543</v>
+        <v>46521</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>46593</v>
+        <v>46541</v>
       </c>
       <c r="F31" t="n">
+        <v>21</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>21 d · ruta crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Electricidad</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>E9</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Conexionado EL — Sector SE#4</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>46500</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>46550</v>
+      </c>
+      <c r="F32" t="n">
         <v>51</v>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>puntas S3 · ruta crítica</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>PRUEBAS · PRECOMISIONADO · COMISIONADO</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>puntas BT+control S4</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pruebas/Comis.</t>
+          <t>Electricidad</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Pruebas Megger EL circuito×circuito</t>
+          <t>Conexionado EL — Terminaciones MT (36 ext.)</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46594</v>
+        <v>46545</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>46614</v>
+        <v>46573</v>
       </c>
       <c r="F33" t="n">
-        <v>21</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
-          <t>513 c · HOLD POINT</t>
+          <t>técnicos cert. ABB</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Pruebas/Comis.</t>
+          <t>Electricidad</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Energización progresiva MT→Transf→BT</t>
+          <t>Conexionado EL — Sector SE#3</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46615</v>
+        <v>46543</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>46631</v>
+        <v>46593</v>
       </c>
       <c r="F34" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1473,45 +1479,23 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>HOLD POINT</t>
+          <t>puntas S3 · ruta crítica</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Pruebas/Comis.</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Precomisionado eléctrico funcional</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="n">
-        <v>46632</v>
-      </c>
-      <c r="E35" s="3" t="n">
-        <v>46652</v>
-      </c>
-      <c r="F35" t="n">
-        <v>21</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>loop check EL + relés</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>PRUEBAS · PRECOMISIONADO · COMISIONADO</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1521,27 +1505,31 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Precomisionado instrumentación (lazos PCS/SIS)</t>
+          <t>Pruebas Megger EL circuito×circuito</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46631</v>
+        <v>46594</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>46660</v>
+        <v>46614</v>
       </c>
       <c r="F36" t="n">
-        <v>30</v>
-      </c>
-      <c r="G36" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>loop check final IN</t>
+          <t>513 c · HOLD POINT</t>
         </is>
       </c>
     </row>
@@ -1553,27 +1541,31 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SAT/Comisionado PCS — Sala INS (Inauco)</t>
+          <t>Energización progresiva MT→Transf→BT</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46463</v>
+        <v>46615</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>46539</v>
+        <v>46631</v>
       </c>
       <c r="F37" t="n">
-        <v>77</v>
-      </c>
-      <c r="G37" t="inlineStr"/>
+        <v>17</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>55 d</t>
+          <t>HOLD POINT</t>
         </is>
       </c>
     </row>
@@ -1585,27 +1577,31 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SAT/Comisionado SIS — HIMA</t>
+          <t>Precomisionado eléctrico funcional</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46463</v>
+        <v>46632</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>46602</v>
+        <v>46652</v>
       </c>
       <c r="F38" t="n">
-        <v>140</v>
-      </c>
-      <c r="G38" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>100 d</t>
+          <t>loop check EL + relés</t>
         </is>
       </c>
     </row>
@@ -1617,31 +1613,27 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Comisionado integrado (EL+PCS+PMS+SIS)</t>
+          <t>Precomisionado instrumentación (lazos PCS/SIS)</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46653</v>
+        <v>46631</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>46740</v>
+        <v>46660</v>
       </c>
       <c r="F39" t="n">
-        <v>88</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>88 d</t>
+          <t>loop check final IN</t>
         </is>
       </c>
     </row>
@@ -1653,27 +1645,27 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>P5</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SAT PMS (HOLD POINT contractual)</t>
+          <t>SAT/Comisionado PCS — Sala INS (Inauco)</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46666</v>
+        <v>46463</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>46726</v>
+        <v>46539</v>
       </c>
       <c r="F40" t="n">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>ventana fija OCT-DIC</t>
+          <t>55 d</t>
         </is>
       </c>
     </row>
@@ -1685,25 +1677,125 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>SAT/Comisionado SIS — HIMA</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>46463</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>46602</v>
+      </c>
+      <c r="F41" t="n">
+        <v>140</v>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>100 d</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Pruebas/Comis.</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Comisionado integrado (EL+PCS+PMS+SIS)</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>46653</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>46740</v>
+      </c>
+      <c r="F42" t="n">
+        <v>88</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>88 d</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Pruebas/Comis.</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SAT PMS (HOLD POINT contractual)</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>46666</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>46726</v>
+      </c>
+      <c r="F43" t="n">
+        <v>61</v>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>ventana fija OCT-DIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Pruebas/Comis.</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>RFSU</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>★★★ RFSU — READY FOR START UP</t>
         </is>
       </c>
-      <c r="D41" s="3" t="n">
+      <c r="D44" s="3" t="n">
         <v>46741</v>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr">
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
         <is>
           <t>SÍ</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>hito gobernante</t>
         </is>

</xml_diff>